<commit_message>
Added Literature Extraction 1 & 2
</commit_message>
<xml_diff>
--- a/research/literature-survey/Literature_Extraction.xlsx
+++ b/research/literature-survey/Literature_Extraction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FraudLens\research\literature-survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C6F1302-11AB-4A9E-AD8E-02945F71FC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFB453E-83FF-437A-87CA-EF83CE41398F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Paper ID</t>
   </si>
@@ -136,6 +136,60 @@
   </si>
   <si>
     <t>http://mdpi.com/2076-3417/12/19/9637</t>
+  </si>
+  <si>
+    <t>P02</t>
+  </si>
+  <si>
+    <t>The Imbalanced Classification of Fraudulent Bank Transactions Using Machine Learning</t>
+  </si>
+  <si>
+    <t>Alexey Ruchay; Elena Feldman; Dmitriy Cherbadzhi; Alexander Sokolov</t>
+  </si>
+  <si>
+    <t>Mathematics, MDPI</t>
+  </si>
+  <si>
+    <t>Detecting fraudulent bank transactions under severe class imbalance</t>
+  </si>
+  <si>
+    <t>To develop and evaluate machine-learning approaches for detecting fraudulent bank transactions and improving classification of the minority fraud class</t>
+  </si>
+  <si>
+    <t>Fraudulent bank/credit-card transactions</t>
+  </si>
+  <si>
+    <t>Data preprocessing; imbalance handling; machine-learning classification; hyperparameter optimization; 10-fold cross-validation</t>
+  </si>
+  <si>
+    <t>Random Forest; TPOT; CatBoost; XGBoost; LightGBM; SVM; KNN; MLP; Decision Tree</t>
+  </si>
+  <si>
+    <t>CreditCardFraud dataset</t>
+  </si>
+  <si>
+    <t>284,807 transactions; 492 fraudulent; 284,315 legitimate</t>
+  </si>
+  <si>
+    <t>Time; Amount; V1–V28 PCA-transformed features; Class label</t>
+  </si>
+  <si>
+    <t>Multiple models achieved high performance; Random Forest reported 0.9999 accuracy, 0.9366 fraud recall and 0.9610 fraud F1</t>
+  </si>
+  <si>
+    <t>The dataset is highly imbalanced and its original feature meanings are unavailable because features are PCA-transformed. The dataset covers only two days of transactions, limiting direct generalization to other financial contexts.</t>
+  </si>
+  <si>
+    <t>Demonstrates the importance of handling class imbalance and evaluating fraud-class Precision, Recall and F1 rather than relying only on Accuracy</t>
+  </si>
+  <si>
+    <t>RQ1; RQ2; RQ3</t>
+  </si>
+  <si>
+    <t>Sections 1, 3.1, 3.2, 4, 5, 6; Table 1; Figure 4</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.3390/math11132862</t>
   </si>
 </sst>
 </file>
@@ -525,11 +579,11 @@
     <col min="11" max="11" width="19.109375" style="3" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="20.21875" style="1" customWidth="1"/>
     <col min="13" max="13" width="27.88671875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="22.109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="22" style="3" customWidth="1"/>
-    <col min="16" max="16" width="21" style="3" customWidth="1"/>
+    <col min="14" max="14" width="35.6640625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="39.109375" style="3" customWidth="1"/>
+    <col min="16" max="16" width="34.5546875" style="3" customWidth="1"/>
     <col min="17" max="17" width="27.33203125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="22.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="35" style="1" customWidth="1"/>
     <col min="19" max="19" width="23.6640625" style="1" customWidth="1"/>
     <col min="20" max="16384" width="8.88671875" style="1"/>
   </cols>
@@ -652,26 +706,64 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
+    <row r="3" spans="1:19" ht="74.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="4">
+        <v>2023</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
@@ -970,7 +1062,9 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="S2" r:id="rId1" xr:uid="{A38B69B3-169A-4791-9FC8-7128EB513ACD}"/>
+    <hyperlink ref="S3" r:id="rId2" xr:uid="{5751E136-023C-4145-B87C-091A39F7EC45}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>